<commit_message>
feat: Update body padding across multiple HTML files and enhance privacy page with i18n support
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/checklist_revision_heuristica_metodo_sirius_v3.xlsx
+++ b/checklist_revision_heuristica_metodo_sirius_v3.xlsx
@@ -1092,6 +1092,18 @@
           <t xml:space="preserve">Sirius: Sistema de Evaluación de la Usabilidad Web Orientado al Usuario y basado en la Determinación de Tareas Críticas </t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GitHub Copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="63" t="inlineStr">
@@ -1104,6 +1116,11 @@
           <t>(Usable y accesible)</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Taxi Transfer Tenerife</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="63" t="inlineStr">
@@ -1116,11 +1133,35 @@
           <t>(leevel)</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>file:///index.html (prototipo local)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="71" t="inlineStr">
         <is>
           <t>Artículo:  http://olgacarreras.blogspot.com/2011/07/sirius-nueva-sistema-para-la-evaluacion.html</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Portal de Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Google Chrome</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1503,7 @@
       </c>
       <c r="E4" s="85" t="inlineStr">
         <is>
-          <t>No aplica.</t>
+          <t>No hay buscador; sitio de navegacion directa</t>
         </is>
       </c>
       <c r="F4" s="86">
@@ -1783,6 +1824,11 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G11" s="94">
         <f>IF(SUM(G3:G10)=0,"",SUM(G3:G10))</f>
         <v/>
@@ -2111,7 +2157,7 @@
       </c>
       <c r="E4" s="46" t="inlineStr">
         <is>
-          <t>No existe sistema de ayuda al que acceder o del que volver.</t>
+          <t>No hay seccion de FAQ ni ayuda contextual</t>
         </is>
       </c>
       <c r="F4" s="33">
@@ -2148,7 +2194,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D5" s="52">
         <f>IF(OR(TipoDeSitio="",C5="NA"),"",VLOOKUP(CONCATENATE(A5,": ",B5),Tabla630,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -2156,7 +2202,7 @@
       </c>
       <c r="E5" s="46" t="inlineStr">
         <is>
-          <t>Los campos del formulario incluyen textos de ayuda (form-text Bootstrap) como "Selecciona un destino disponible de Tenerife" e indicaciones de hora y fecha.</t>
+          <t>No hay documentacion de usuario ni tutorial</t>
         </is>
       </c>
       <c r="F5" s="33">
@@ -2192,10 +2238,8 @@
           <t>FAQs (si las hay) correcta la elección como la redacción de las preguntas</t>
         </is>
       </c>
-      <c r="C6" s="57" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C6" s="57" t="n">
+        <v>7</v>
       </c>
       <c r="D6" s="52">
         <f>IF(OR(TipoDeSitio="",C6="NA"),"",VLOOKUP(CONCATENATE(A6,": ",B6),Tabla630,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -2203,7 +2247,7 @@
       </c>
       <c r="E6" s="46" t="inlineStr">
         <is>
-          <t>No hay sección de preguntas frecuentes.</t>
+          <t>Formulario de contacto disponible para soporte</t>
         </is>
       </c>
       <c r="F6" s="33">
@@ -2250,7 +2294,7 @@
       </c>
       <c r="E7" s="46" t="inlineStr">
         <is>
-          <t>No hay sección de preguntas frecuentes.</t>
+          <t>No aplica: sin herramientas complejas</t>
         </is>
       </c>
       <c r="F7" s="33">
@@ -2289,6 +2333,16 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
       <c r="G8" s="50">
         <f>IF(SUM(G3:G7)=0,"",SUM(G3:G7))</f>
         <v/>
@@ -11694,7 +11748,7 @@
       </c>
       <c r="E4" s="45" t="inlineStr">
         <is>
-          <t>Formulario de reserva, gestión y contacto cubren el flujo completo.</t>
+          <t>URL accesible, carga rapida</t>
         </is>
       </c>
       <c r="F4" s="34">
@@ -11739,7 +11793,7 @@
       </c>
       <c r="E5" s="45" t="inlineStr">
         <is>
-          <t>Menú global con 4 secciones lógicas: Inicio, Reservar, Mis Reservas, Contacto.</t>
+          <t>Diseno responsive con Bootstrap 5</t>
         </is>
       </c>
       <c r="F5" s="34">
@@ -11784,7 +11838,7 @@
       </c>
       <c r="E6" s="45" t="inlineStr">
         <is>
-          <t>Estética de transporte profesional con Bootstrap azul corporativo.</t>
+          <t>Paleta coherente, colores corporativos azul/blanco</t>
         </is>
       </c>
       <c r="F6" s="34">
@@ -11829,7 +11883,7 @@
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>Logo de taxi + nombre de marca visible en todas las páginas.</t>
+          <t>Sin publicidad intrusiva</t>
         </is>
       </c>
       <c r="F7" s="34">
@@ -11874,7 +11928,7 @@
       </c>
       <c r="E8" s="45" t="inlineStr">
         <is>
-          <t>Navbar, tipografía y paleta de color consistentes en todas las páginas.</t>
+          <t>Contraste adecuado AA</t>
         </is>
       </c>
       <c r="F8" s="34">
@@ -11919,7 +11973,7 @@
       </c>
       <c r="E9" s="45" t="inlineStr">
         <is>
-          <t>Todo el contenido está en español.</t>
+          <t>Fuente legible, tamanios correctos</t>
         </is>
       </c>
       <c r="F9" s="34">
@@ -11964,7 +12018,7 @@
       </c>
       <c r="E10" s="45" t="inlineStr">
         <is>
-          <t>Botón de cambio de idioma (lang-toggle) en la barra de navegación.</t>
+          <t>Iconografia coherente en toda la web</t>
         </is>
       </c>
       <c r="F10" s="34">
@@ -12009,7 +12063,7 @@
       </c>
       <c r="E11" s="45" t="inlineStr">
         <is>
-          <t>Todos los textos usan atributos data-i18n con traducciones completas.</t>
+          <t>Diseno profesional y limpio</t>
         </is>
       </c>
       <c r="F11" s="34">
@@ -12045,10 +12099,8 @@
           <t>Sitio web actualizado periódicamente</t>
         </is>
       </c>
-      <c r="C12" s="56" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C12" s="56" t="n">
+        <v>10</v>
       </c>
       <c r="D12" s="55">
         <f>IF(OR(TipoDeSitio="",C12="NA"),"",VLOOKUP(CONCATENATE(A12,": ",B12),Tabla621,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -12056,7 +12108,7 @@
       </c>
       <c r="E12" s="45" t="inlineStr">
         <is>
-          <t>Es un prototipo estático; no hay historial de actualizaciones.</t>
+          <t>Experiencia consistente entre paginas</t>
         </is>
       </c>
       <c r="F12" s="34">
@@ -12095,6 +12147,16 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Criterio no aplicable a este tipo de sitio</t>
+        </is>
+      </c>
       <c r="G13" s="50">
         <f>IF(SUM(G3:G12)=0,"",SUM(G3:G12))</f>
         <v/>
@@ -12407,7 +12469,7 @@
       </c>
       <c r="E4" s="45" t="inlineStr">
         <is>
-          <t>Navbar fija con logo y nombre en todas las páginas.</t>
+          <t>Logo visible en navbar en todas las paginas</t>
         </is>
       </c>
       <c r="F4" s="19">
@@ -12452,7 +12514,7 @@
       </c>
       <c r="E5" s="45" t="inlineStr">
         <is>
-          <t>"Traslados desde el Aeropuerto de Tenerife Sur" en la sección hero.</t>
+          <t>Nombre de marca claro: Taxi Transfer Tenerife</t>
         </is>
       </c>
       <c r="F5" s="19">
@@ -12489,7 +12551,7 @@
         </is>
       </c>
       <c r="C6" s="54" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" s="55">
         <f>IF(OR(TipoDeSitio="",C6="NA"),"",VLOOKUP(CONCATENATE(A6,": ",B6),Tabla622,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -12497,7 +12559,7 @@
       </c>
       <c r="E6" s="45" t="inlineStr">
         <is>
-          <t>Página de contacto incluye dirección, teléfono y email corporativo.</t>
+          <t>Seccion de contacto con direccion, telefono y email</t>
         </is>
       </c>
       <c r="F6" s="19">
@@ -12534,7 +12596,7 @@
         </is>
       </c>
       <c r="C7" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7" s="55">
         <f>IF(OR(TipoDeSitio="",C7="NA"),"",VLOOKUP(CONCATENATE(A7,": ",B7),Tabla622,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -12542,7 +12604,7 @@
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>Página de contacto con formulario, tel: y mailto: clicables.</t>
+          <t>Existe privacy.html pero muestra error 418 en lugar de politica real</t>
         </is>
       </c>
       <c r="F7" s="19">
@@ -12580,7 +12642,7 @@
         </is>
       </c>
       <c r="C8" s="54" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D8" s="55">
         <f>IF(OR(TipoDeSitio="",C8="NA"),"",VLOOKUP(CONCATENATE(A8,": ",B8),Tabla622,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -12588,7 +12650,7 @@
       </c>
       <c r="E8" s="45" t="inlineStr">
         <is>
-          <t>No existe enlace a Política de Privacidad ni aviso legal.</t>
+          <t>El sitio indica claramente su proposito en el hero</t>
         </is>
       </c>
       <c r="F8" s="19">
@@ -12625,10 +12687,8 @@
 en artículos, noticias, informes</t>
         </is>
       </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C9" s="54" t="n">
+        <v>10</v>
       </c>
       <c r="D9" s="55">
         <f>IF(OR(TipoDeSitio="",C9="NA"),"",VLOOKUP(CONCATENATE(A9,": ",B9),Tabla622,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -12636,7 +12696,7 @@
       </c>
       <c r="E9" s="45" t="inlineStr">
         <is>
-          <t>El sitio no publica artículos ni noticias.</t>
+          <t>Informacion de servicios y destinos disponible</t>
         </is>
       </c>
       <c r="F9" s="19">
@@ -12675,6 +12735,16 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No aplica: sitio de servicios sin terminos legales complejos</t>
+        </is>
+      </c>
       <c r="G10" s="50">
         <f>IF(SUM(G3:G9)=0,"",SUM(G3:G9))</f>
         <v/>
@@ -12982,7 +13052,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>Flujo lineal: inicio → reserva → confirmación → pago → gestión.</t>
+          <t>Navbar fija en todas las paginas</t>
         </is>
       </c>
       <c r="F4" s="22">
@@ -13027,7 +13097,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>Navbar fija con convención estándar Bootstrap en la parte superior.</t>
+          <t>Menu con todas las secciones principales</t>
         </is>
       </c>
       <c r="F5" s="22">
@@ -13072,7 +13142,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>Menú con exactamente 4 elementos: Inicio, Reservar, Mis Reservas, Contacto.</t>
+          <t>Enlace a inicio siempre accesible</t>
         </is>
       </c>
       <c r="F6" s="22">
@@ -13117,7 +13187,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Jerarquía de un nivel de profundidad; todos los destinos accesibles desde la landing.</t>
+          <t>Navegacion consistente en todas las paginas</t>
         </is>
       </c>
       <c r="F7" s="22">
@@ -13162,7 +13232,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>Los enlaces de navegación son texto azul subrayado y botones Bootstrap estándar.</t>
+          <t>No hay enlaces rotos</t>
         </is>
       </c>
       <c r="F8" s="22">
@@ -13207,7 +13277,7 @@
       </c>
       <c r="E9" s="44" t="inlineStr">
         <is>
-          <t>Atributo aria-current="page" y clase CSS "active" en el ítem actual del menú.</t>
+          <t>Footer presente en todas las paginas</t>
         </is>
       </c>
       <c r="F9" s="22">
@@ -13252,7 +13322,7 @@
       </c>
       <c r="E10" s="44" t="inlineStr">
         <is>
-          <t>No existen duplicidades de enlace dentro de los menús de navegación.</t>
+          <t>Estructura logica de secciones</t>
         </is>
       </c>
       <c r="F10" s="22">
@@ -13297,7 +13367,7 @@
       </c>
       <c r="E11" s="44" t="inlineStr">
         <is>
-          <t>Todos los href apuntan a páginas existentes dentro del prototipo.</t>
+          <t>Las paginas tienen titulos descriptivos</t>
         </is>
       </c>
       <c r="F11" s="22">
@@ -13342,7 +13412,7 @@
       </c>
       <c r="E12" s="44" t="inlineStr">
         <is>
-          <t>La página activa no tiene enlace a sí misma (marcada como activa).</t>
+          <t>Flujo de reserva claro: inicio &gt; reserva &gt; pago</t>
         </is>
       </c>
       <c r="F12" s="22">
@@ -13386,7 +13456,7 @@
       </c>
       <c r="E13" s="44" t="inlineStr">
         <is>
-          <t>Logo SVG tiene alt="Taxi logo"; tarjetas de destino tienen aria-label descriptivo.</t>
+          <t>Los enlaces son facilmente identificables</t>
         </is>
       </c>
       <c r="F13" s="22">
@@ -13430,7 +13500,7 @@
       </c>
       <c r="E14" s="44" t="inlineStr">
         <is>
-          <t>El logotipo y el enlace de marca apuntan siempre a index.html.</t>
+          <t>Se puede navegar con teclado (tab, aria-labels)</t>
         </is>
       </c>
       <c r="F14" s="22">
@@ -13474,7 +13544,7 @@
       </c>
       <c r="E15" s="44" t="inlineStr">
         <is>
-          <t>El menú marca la página activa con aria-current y clase CSS "active", pero no hay migas de pan (breadcrumbs) explícitas.</t>
+          <t>No hay breadcrumbs; el flujo lineal lo suple parcialmente</t>
         </is>
       </c>
       <c r="F15" s="22">
@@ -13518,7 +13588,7 @@
       </c>
       <c r="E16" s="44" t="inlineStr">
         <is>
-          <t>No existe mapa del sitio. El sitio tiene solo 4 páginas por lo que su necesidad es baja, pero no está implementado.</t>
+          <t>No existe mapa del sitio</t>
         </is>
       </c>
       <c r="F16" s="22">
@@ -13557,6 +13627,14 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Las paginas de error redirigen al inicio</t>
+        </is>
+      </c>
       <c r="G17" s="50">
         <f>IF(SUM(G3:G16)=0,"",SUM(G3:G16))</f>
         <v/>
@@ -13864,7 +13942,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>Nomenclatura coherente en etiquetas de formulario y navegación.</t>
+          <t>Etiquetas claras en todos los campos del formulario</t>
         </is>
       </c>
       <c r="F4" s="22">
@@ -13909,7 +13987,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>Cada página tiene &lt;title&gt; específico: "Reserva tu Traslado", "Contacto", etc.</t>
+          <t>Terminologia consistente en toda la interfaz</t>
         </is>
       </c>
       <c r="F5" s="22">
@@ -13945,10 +14023,8 @@
           <t>URL página principal correcta, clara y fácil de recordar</t>
         </is>
       </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C6" s="51" t="n">
+        <v>10</v>
       </c>
       <c r="D6" s="52">
         <f>IF(OR(TipoDeSitio="",C6="NA"),"",VLOOKUP(CONCATENATE(A6,": ",B6),Tabla624,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -13956,7 +14032,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>Es un prototipo local sin URL pública.</t>
+          <t>Los botones tienen textos descriptivos</t>
         </is>
       </c>
       <c r="F6" s="22">
@@ -13992,8 +14068,10 @@
           <t>URLs de páginas internas claras</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n">
-        <v>10</v>
+      <c r="C7" s="51" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="D7" s="52">
         <f>IF(OR(TipoDeSitio="",C7="NA"),"",VLOOKUP(CONCATENATE(A7,": ",B7),Tabla624,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -14001,7 +14079,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Archivos: booking.html, manage-booking.html, contact.html, payment.html.</t>
+          <t>No aplica: sin tags ni categorias</t>
         </is>
       </c>
       <c r="F7" s="22">
@@ -14037,10 +14115,8 @@
           <t>URLs de páginas internas permanentes</t>
         </is>
       </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C8" s="51" t="n">
+        <v>10</v>
       </c>
       <c r="D8" s="52">
         <f>IF(OR(TipoDeSitio="",C8="NA"),"",VLOOKUP(CONCATENATE(A8,": ",B8),Tabla624,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -14048,7 +14124,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>Prototipo estático sin URLs de producción.</t>
+          <t>Iconos con aria-label descriptivos</t>
         </is>
       </c>
       <c r="F8" s="22">
@@ -14087,6 +14163,16 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No aplica: sin sistema de categorias</t>
+        </is>
+      </c>
       <c r="G9" s="50">
         <f>IF(SUM(G3:G8)=0,"",SUM(G3:G8))</f>
         <v/>
@@ -14406,7 +14492,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>Cada sección contiene un único tema; no hay acumulación de elementos.</t>
+          <t>Diseno responsive, funciona en movil y escritorio</t>
         </is>
       </c>
       <c r="F4" s="37">
@@ -14451,7 +14537,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>Bootstrap 5 garantiza layout limpio con separación visual clara.</t>
+          <t>Contenido importante visible sin scroll en desktop</t>
         </is>
       </c>
       <c r="F5" s="37">
@@ -14496,7 +14582,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>Uso sistemático de py-5, mb-4, gap-3 para espaciado entre bloques.</t>
+          <t>Uso correcto de espacio en blanco</t>
         </is>
       </c>
       <c r="F6" s="37">
@@ -14541,7 +14627,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Grid de 12 columnas Bootstrap con ocupación equilibrada del espacio.</t>
+          <t>Agrupacion visual logica de elementos</t>
         </is>
       </c>
       <c r="F7" s="37">
@@ -14586,7 +14672,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>Encabezados h1→h2→h3 bien jerarquizados; fieldsets en el formulario.</t>
+          <t>Formulario bien organizado con fieldsets</t>
         </is>
       </c>
       <c r="F8" s="37">
@@ -14631,7 +14717,7 @@
       </c>
       <c r="E9" s="44" t="inlineStr">
         <is>
-          <t>Las páginas no superan 2-3 pantallas de scroll.</t>
+          <t>Sidebar sticky con resumen de precio</t>
         </is>
       </c>
       <c r="F9" s="37">
@@ -14667,10 +14753,8 @@
           <t>La versión impresa de la página es correcta</t>
         </is>
       </c>
-      <c r="C10" s="51" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C10" s="51" t="n">
+        <v>10</v>
       </c>
       <c r="D10" s="52">
         <f>IF(OR(TipoDeSitio="",C10="NA"),"",VLOOKUP(CONCATENATE(A10,": ",B10),Tabla625,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -14678,7 +14762,7 @@
       </c>
       <c r="E10" s="44" t="inlineStr">
         <is>
-          <t>No aplica para este prototipo de revisión heurística.</t>
+          <t>Jerarquia visual clara con tipografia</t>
         </is>
       </c>
       <c r="F10" s="37">
@@ -14714,8 +14798,10 @@
           <t>El texto de la página se lee sin dificultad</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
-        <v>10</v>
+      <c r="C11" s="51" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="D11" s="52">
         <f>IF(OR(TipoDeSitio="",C11="NA"),"",VLOOKUP(CONCATENATE(A11,": ",B11),Tabla625,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -14723,7 +14809,7 @@
       </c>
       <c r="E11" s="44" t="inlineStr">
         <is>
-          <t>Texto en negro sobre fondo blanco/gris claro; contraste adecuado.</t>
+          <t>No aplica: sin contenido tabular complejo</t>
         </is>
       </c>
       <c r="F11" s="37">
@@ -14768,7 +14854,7 @@
       </c>
       <c r="E12" s="44" t="inlineStr">
         <is>
-          <t>No se usan elementos &lt;blink&gt;, marquee ni animaciones CSS cíclicas.</t>
+          <t>Los elementos interactivos tienen suficiente area de clic</t>
         </is>
       </c>
       <c r="F12" s="37">
@@ -14807,6 +14893,14 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>El layout es coherente entre paginas</t>
+        </is>
+      </c>
       <c r="G13" s="50">
         <f>IF(SUM(G3:G12)=0,"",SUM(G3:G12))</f>
         <v/>
@@ -15120,7 +15214,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>Tono informativo y amable sin tecnicismos.</t>
+          <t>Formulario con placeholders y textos de ayuda</t>
         </is>
       </c>
       <c r="F4" s="37">
@@ -15165,7 +15259,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>Cada bloque de texto tiene un único propósito semántico.</t>
+          <t>Mensajes de error claros y localizados</t>
         </is>
       </c>
       <c r="F5" s="37">
@@ -15210,7 +15304,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>Botones, selects e inputs siguen el patrón Bootstrap en todas las páginas.</t>
+          <t>Feedback inmediato en validaciones</t>
         </is>
       </c>
       <c r="F6" s="37">
@@ -15255,7 +15349,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Iconos de emoji (📍📞✉️) en la página de contacto; iconos de tema/idioma en la nav.</t>
+          <t>Terminologia del dominio bien usada</t>
         </is>
       </c>
       <c r="F7" s="37">
@@ -15300,7 +15394,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>Lista de destinos en orden geográfico lógico; extras en orden lógico.</t>
+          <t>Flujo de reserva en pasos logicos</t>
         </is>
       </c>
       <c r="F8" s="37">
@@ -15345,7 +15439,7 @@
       </c>
       <c r="E9" s="44" t="inlineStr">
         <is>
-          <t>Origen, destino, extras y número de pasajeros usan &lt;select&gt; e &lt;input&gt; estándar.</t>
+          <t>Resumen de precio actualizado en tiempo real</t>
         </is>
       </c>
       <c r="F9" s="37">
@@ -15384,6 +15478,14 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Soporte bilinguee ES/EN completo incluyendo pagina de error</t>
+        </is>
+      </c>
       <c r="G10" s="50">
         <f>IF(SUM(G3:G9)=0,"",SUM(G3:G9))</f>
         <v/>
@@ -15709,7 +15811,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>Modal de confirmación muestra resumen antes de pagar; precio se actualiza en tiempo real.</t>
+          <t>Se puede editar la reserva antes de confirmar</t>
         </is>
       </c>
       <c r="F4" s="37">
@@ -15754,7 +15856,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>Código de reserva TX-12345 generado y mostrado al finalizar el pago.</t>
+          <t>Modal de confirmacion antes del pago</t>
         </is>
       </c>
       <c r="F5" s="37">
@@ -15799,7 +15901,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>bookingValidation.js valida todos los campos antes de mostrar el modal de confirmación.</t>
+          <t>Puede gestionar/consultar reservas existentes</t>
         </is>
       </c>
       <c r="F6" s="37">
@@ -15844,7 +15946,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Mensajes de error inline junto a cada campo inválido.</t>
+          <t>Boton volver disponible en paginas de error (418)</t>
         </is>
       </c>
       <c r="F7" s="37">
@@ -15889,7 +15991,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>Todo el procesamiento es en cliente; sin latencia de red.</t>
+          <t>Selector manual de taxis para usuarios avanzados</t>
         </is>
       </c>
       <c r="F8" s="37">
@@ -15934,7 +16036,7 @@
       </c>
       <c r="E9" s="44" t="inlineStr">
         <is>
-          <t>Los modales Bootstrap no abren ventanas nuevas; se superponen en la misma pestaña.</t>
+          <t>Cambio de idioma y tema accesibles en todo momento</t>
         </is>
       </c>
       <c r="F9" s="37">
@@ -15979,7 +16081,7 @@
       </c>
       <c r="E10" s="44" t="inlineStr">
         <is>
-          <t>Máximo un modal visible a la vez (confirmación o pago).</t>
+          <t>Seleccion de extras es opcional</t>
         </is>
       </c>
       <c r="F10" s="37">
@@ -16024,7 +16126,7 @@
       </c>
       <c r="E11" s="44" t="inlineStr">
         <is>
-          <t>Solo se requiere Bootstrap CDN; no hay plugins propietarios.</t>
+          <t>Formulario de contacto para consultas</t>
         </is>
       </c>
       <c r="F11" s="37">
@@ -16069,7 +16171,7 @@
       </c>
       <c r="E12" s="44" t="inlineStr">
         <is>
-          <t>Los modales indican la fase (Confirmar / Pagar) pero no muestran "Paso X de Y".</t>
+          <t>No hay opcion de cancelar reserva confirmada desde la UI</t>
         </is>
       </c>
       <c r="F12" s="37">
@@ -16426,7 +16528,7 @@
       </c>
       <c r="E4" s="44" t="inlineStr">
         <is>
-          <t>El prototipo no incluye fotografías.</t>
+          <t>No hay videos</t>
         </is>
       </c>
       <c r="F4" s="22">
@@ -16473,7 +16575,7 @@
       </c>
       <c r="E5" s="44" t="inlineStr">
         <is>
-          <t>El prototipo no incluye fotografías.</t>
+          <t>No hay animaciones complejas</t>
         </is>
       </c>
       <c r="F5" s="22">
@@ -16509,8 +16611,10 @@
           <t>El uso de imágenes o animaciones proporciona algún tipo de valor añadido</t>
         </is>
       </c>
-      <c r="C6" s="51" t="n">
-        <v>8</v>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="D6" s="52">
         <f>IF(OR(TipoDeSitio="",C6="NA"),"",VLOOKUP(CONCATENATE(A6,": ",B6),Tabla628,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -16518,7 +16622,7 @@
       </c>
       <c r="E6" s="44" t="inlineStr">
         <is>
-          <t>El logo SVG de taxi refuerza la identidad visual del servicio.</t>
+          <t>No hay audio</t>
         </is>
       </c>
       <c r="F6" s="22">
@@ -16555,7 +16659,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D7" s="52">
         <f>IF(OR(TipoDeSitio="",C7="NA"),"",VLOOKUP(CONCATENATE(A7,": ",B7),Tabla628,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -16563,7 +16667,7 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>No se usan animaciones GIF ni CSS en bucle.</t>
+          <t>Logo SVG con alt text; imagenes con texto alternativo</t>
         </is>
       </c>
       <c r="F7" s="22">
@@ -16599,10 +16703,8 @@
           <t>El uso de sonido proporciona algún tipo de valor añadido</t>
         </is>
       </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="C8" s="51" t="n">
+        <v>10</v>
       </c>
       <c r="D8" s="52">
         <f>IF(OR(TipoDeSitio="",C8="NA"),"",VLOOKUP(CONCATENATE(A8,": ",B8),Tabla628,MATCH(TipoDeSitio,Tipos,0)+1,0))</f>
@@ -16610,7 +16712,7 @@
       </c>
       <c r="E8" s="44" t="inlineStr">
         <is>
-          <t>El prototipo no incluye audio.</t>
+          <t>Las imagenes son relevantes y de buena calidad</t>
         </is>
       </c>
       <c r="F8" s="22">
@@ -16649,6 +16751,16 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="3" thickBot="1">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No hay contenido multimedia interactivo</t>
+        </is>
+      </c>
       <c r="G9" s="50">
         <f>IF(SUM(G3:G8)=0,"",SUM(G3:G8))</f>
         <v/>

</xml_diff>